<commit_message>
Release v2.7.0 alpha fieldwork modules
</commit_message>
<xml_diff>
--- a/app/src/main/assets/methodmesh/odk_templates/conversationtranslate/example_odk_showcase_conversation_translate.xlsx
+++ b/app/src/main/assets/methodmesh/odk_templates/conversationtranslate/example_odk_showcase_conversation_translate.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="survey" sheetId="1" r:id="R52027d3377ad4629"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="choices" sheetId="2" r:id="R70216516a5294d45"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="settings" sheetId="3" r:id="Rc993aeab6a674d83"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="survey" sheetId="1" r:id="R0cd6889faf084afe"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="choices" sheetId="2" r:id="Rf47e7a93e51e4c43"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="settings" sheetId="3" r:id="R09de356e085749e6"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -46,7 +46,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="10">
+  <x:cellXfs count="11">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -65,6 +65,7 @@
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -334,17 +335,17 @@
         <x:v>MethodMesh Conversation translator — conversation.translate</x:v>
       </x:c>
       <x:c r="D2" s="8" t="str">
-        <x:v>Run a bilingual speech translation session</x:v>
-      </x:c>
-      <x:c r="E2" s="8" t="str"/>
-      <x:c r="F2" s="8" t="str"/>
-      <x:c r="G2" s="8" t="str"/>
-      <x:c r="H2" s="8" t="str"/>
-      <x:c r="I2" s="8" t="str"/>
-      <x:c r="J2" s="8" t="str"/>
-      <x:c r="K2" s="8" t="str"/>
-      <x:c r="L2" s="8" t="str"/>
-      <x:c r="M2" s="8" t="str"/>
+        <x:v>Two-person live translation with flag-first participant language choice and pauseable transcript.</x:v>
+      </x:c>
+      <x:c r="E2" s="8"/>
+      <x:c r="F2" s="8"/>
+      <x:c r="G2" s="8"/>
+      <x:c r="H2" s="8"/>
+      <x:c r="I2" s="8"/>
+      <x:c r="J2" s="8"/>
+      <x:c r="K2" s="8"/>
+      <x:c r="L2" s="8"/>
+      <x:c r="M2" s="8"/>
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="8" t="str">
@@ -357,20 +358,20 @@
         <x:v>Run conversation.translate</x:v>
       </x:c>
       <x:c r="D3" s="8" t="str">
-        <x:v>This form invokes only this MethodMesh capability. Inputs shown here are only those relevant to this call; capability interaction may continue in the native MethodMesh surface and return on Commit.</x:v>
+        <x:v>Native participant UI opens in MethodMesh.</x:v>
       </x:c>
       <x:c r="E3" s="8" t="str">
         <x:v>field-list</x:v>
       </x:c>
-      <x:c r="F3" s="8" t="str"/>
-      <x:c r="G3" s="8" t="str"/>
-      <x:c r="H3" s="8" t="str"/>
-      <x:c r="I3" s="8" t="str"/>
-      <x:c r="J3" s="8" t="str"/>
-      <x:c r="K3" s="8" t="str"/>
-      <x:c r="L3" s="8" t="str"/>
+      <x:c r="F3" s="8"/>
+      <x:c r="G3" s="8"/>
+      <x:c r="H3" s="8"/>
+      <x:c r="I3" s="8"/>
+      <x:c r="J3" s="8"/>
+      <x:c r="K3" s="8"/>
+      <x:c r="L3" s="8"/>
       <x:c r="M3" s="8" t="str">
-        <x:v>com.example.methodmesh.EXECUTE_METHOD(method_id='conversation.translate',input_language_a=${language_a_input},input_language_b=${language_b_input},input_spoken_output=${spoken_output_input},input_prefer_offline=${prefer_offline_input},input_payload_mode='FULL',return_mode='flat')</x:v>
+        <x:v>com.example.methodmesh.EXECUTE_METHOD(method_id='conversation.translate',input_language_a=${language_a_input},input_language_b=${language_b_input},input_arabic_variant_a=${arabic_variant_a_input},input_arabic_variant_b=${arabic_variant_b_input},input_voice_a=${voice_a_input},input_voice_b=${voice_b_input},input_transcript_on_start=${transcript_on_start_input},input_spoken_output=${spoken_output_input},input_prefer_offline=${prefer_offline_input},input_payload_mode='FULL',return_mode='flat')</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
@@ -384,246 +385,383 @@
         <x:v>First language</x:v>
       </x:c>
       <x:c r="D4" s="8" t="str">
-        <x:v>Download the language pack in MethodMesh settings before offline use.</x:v>
-      </x:c>
-      <x:c r="E4" s="8" t="str"/>
+        <x:v>Participant can change this by flag in MethodMesh.</x:v>
+      </x:c>
+      <x:c r="E4" s="8"/>
       <x:c r="F4" s="8" t="str">
         <x:v>yes</x:v>
       </x:c>
-      <x:c r="G4" s="8" t="str"/>
-      <x:c r="H4" s="8" t="str"/>
-      <x:c r="I4" s="8" t="str"/>
-      <x:c r="J4" s="8" t="str"/>
+      <x:c r="G4" s="8"/>
+      <x:c r="H4" s="8"/>
+      <x:c r="I4" s="8"/>
+      <x:c r="J4" s="8"/>
       <x:c r="K4" s="8" t="str">
         <x:v>en</x:v>
       </x:c>
-      <x:c r="L4" s="8" t="str"/>
-      <x:c r="M4" s="8" t="str"/>
+      <x:c r="L4" s="8"/>
+      <x:c r="M4" s="8"/>
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="8" t="str">
-        <x:v>select_one language</x:v>
+        <x:v>select_one arabic_variant</x:v>
       </x:c>
       <x:c r="B5" s="8" t="str">
-        <x:v>language_b_input</x:v>
+        <x:v>arabic_variant_a_input</x:v>
       </x:c>
       <x:c r="C5" s="8" t="str">
-        <x:v>Second language</x:v>
+        <x:v>Arabic speech variant A</x:v>
       </x:c>
       <x:c r="D5" s="8" t="str">
-        <x:v>Download the language pack in MethodMesh settings before offline use.</x:v>
-      </x:c>
-      <x:c r="E5" s="8" t="str"/>
+        <x:v>Shown only for Arabic; affects speech recognition/TTS, not ML Kit translation.</x:v>
+      </x:c>
+      <x:c r="E5" s="8"/>
       <x:c r="F5" s="8" t="str">
         <x:v>yes</x:v>
       </x:c>
-      <x:c r="G5" s="8" t="str"/>
-      <x:c r="H5" s="8" t="str"/>
-      <x:c r="I5" s="8" t="str"/>
-      <x:c r="J5" s="8" t="str"/>
+      <x:c r="G5" s="8" t="str">
+        <x:v>${language_a_input} = 'ar'</x:v>
+      </x:c>
+      <x:c r="H5" s="8"/>
+      <x:c r="I5" s="8"/>
+      <x:c r="J5" s="8"/>
       <x:c r="K5" s="8" t="str">
-        <x:v>es</x:v>
-      </x:c>
-      <x:c r="L5" s="8" t="str"/>
-      <x:c r="M5" s="8" t="str"/>
+        <x:v>gulf</x:v>
+      </x:c>
+      <x:c r="L5" s="8"/>
+      <x:c r="M5" s="8"/>
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="8" t="str">
-        <x:v>select_one yes_no</x:v>
+        <x:v>select_one voice_preference</x:v>
       </x:c>
       <x:c r="B6" s="8" t="str">
-        <x:v>spoken_output_input</x:v>
+        <x:v>voice_a_input</x:v>
       </x:c>
       <x:c r="C6" s="8" t="str">
-        <x:v>Speak translations aloud</x:v>
-      </x:c>
-      <x:c r="D6" s="8" t="str"/>
-      <x:c r="E6" s="8" t="str"/>
+        <x:v>Speaker A voice</x:v>
+      </x:c>
+      <x:c r="D6" s="8" t="str">
+        <x:v>Female/male TTS preference; actual availability depends on the installed Android voice engine.</x:v>
+      </x:c>
+      <x:c r="E6" s="8"/>
       <x:c r="F6" s="8" t="str">
         <x:v>yes</x:v>
       </x:c>
-      <x:c r="G6" s="8" t="str"/>
-      <x:c r="H6" s="8" t="str"/>
-      <x:c r="I6" s="8" t="str"/>
-      <x:c r="J6" s="8" t="str"/>
+      <x:c r="G6" s="8"/>
+      <x:c r="H6" s="8"/>
+      <x:c r="I6" s="8"/>
+      <x:c r="J6" s="8"/>
       <x:c r="K6" s="8" t="str">
-        <x:v>true</x:v>
-      </x:c>
-      <x:c r="L6" s="8" t="str"/>
-      <x:c r="M6" s="8" t="str"/>
+        <x:v>female</x:v>
+      </x:c>
+      <x:c r="L6" s="8"/>
+      <x:c r="M6" s="8"/>
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="8" t="str">
-        <x:v>select_one yes_no</x:v>
+        <x:v>select_one language</x:v>
       </x:c>
       <x:c r="B7" s="8" t="str">
-        <x:v>prefer_offline_input</x:v>
+        <x:v>language_b_input</x:v>
       </x:c>
       <x:c r="C7" s="8" t="str">
-        <x:v>Prefer offline speech recognition</x:v>
-      </x:c>
-      <x:c r="D7" s="8" t="str"/>
-      <x:c r="E7" s="8" t="str"/>
+        <x:v>Second language</x:v>
+      </x:c>
+      <x:c r="D7" s="8" t="str">
+        <x:v>Participant can change this by flag in MethodMesh.</x:v>
+      </x:c>
+      <x:c r="E7" s="8"/>
       <x:c r="F7" s="8" t="str">
         <x:v>yes</x:v>
       </x:c>
-      <x:c r="G7" s="8" t="str"/>
-      <x:c r="H7" s="8" t="str"/>
-      <x:c r="I7" s="8" t="str"/>
-      <x:c r="J7" s="8" t="str"/>
+      <x:c r="G7" s="8"/>
+      <x:c r="H7" s="8"/>
+      <x:c r="I7" s="8"/>
+      <x:c r="J7" s="8"/>
       <x:c r="K7" s="8" t="str">
-        <x:v>true</x:v>
-      </x:c>
-      <x:c r="L7" s="8" t="str"/>
-      <x:c r="M7" s="8" t="str"/>
+        <x:v>es</x:v>
+      </x:c>
+      <x:c r="L7" s="8"/>
+      <x:c r="M7" s="8"/>
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="8" t="str">
-        <x:v>text</x:v>
+        <x:v>select_one arabic_variant</x:v>
       </x:c>
       <x:c r="B8" s="8" t="str">
-        <x:v>methodmesh_execution_id</x:v>
+        <x:v>arabic_variant_b_input</x:v>
       </x:c>
       <x:c r="C8" s="8" t="str">
-        <x:v>MethodMesh execution ID</x:v>
+        <x:v>Arabic speech variant B</x:v>
       </x:c>
       <x:c r="D8" s="8" t="str">
-        <x:v>Returned by MethodMesh.</x:v>
-      </x:c>
-      <x:c r="E8" s="8" t="str">
-        <x:v>hidden-answer</x:v>
-      </x:c>
-      <x:c r="F8" s="8" t="str"/>
-      <x:c r="G8" s="8" t="str"/>
-      <x:c r="H8" s="8" t="str"/>
-      <x:c r="I8" s="8" t="str"/>
-      <x:c r="J8" s="8" t="str"/>
-      <x:c r="K8" s="8" t="str"/>
-      <x:c r="L8" s="8" t="str">
+        <x:v>Shown only for Arabic; affects speech recognition/TTS, not ML Kit translation.</x:v>
+      </x:c>
+      <x:c r="E8" s="8"/>
+      <x:c r="F8" s="8" t="str">
         <x:v>yes</x:v>
       </x:c>
-      <x:c r="M8" s="8" t="str"/>
+      <x:c r="G8" s="8" t="str">
+        <x:v>${language_b_input} = 'ar'</x:v>
+      </x:c>
+      <x:c r="H8" s="8"/>
+      <x:c r="I8" s="8"/>
+      <x:c r="J8" s="8"/>
+      <x:c r="K8" s="8" t="str">
+        <x:v>gulf</x:v>
+      </x:c>
+      <x:c r="L8" s="8"/>
+      <x:c r="M8" s="8"/>
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="8" t="str">
-        <x:v>text</x:v>
+        <x:v>select_one voice_preference</x:v>
       </x:c>
       <x:c r="B9" s="8" t="str">
-        <x:v>methodmesh_status</x:v>
+        <x:v>voice_b_input</x:v>
       </x:c>
       <x:c r="C9" s="8" t="str">
-        <x:v>MethodMesh status</x:v>
+        <x:v>Speaker B voice</x:v>
       </x:c>
       <x:c r="D9" s="8" t="str">
-        <x:v>Shared MethodMesh transport status, where projected by the runtime.</x:v>
-      </x:c>
-      <x:c r="E9" s="8" t="str">
-        <x:v>hidden-answer</x:v>
-      </x:c>
-      <x:c r="F9" s="8" t="str"/>
-      <x:c r="G9" s="8" t="str"/>
-      <x:c r="H9" s="8" t="str"/>
-      <x:c r="I9" s="8" t="str"/>
-      <x:c r="J9" s="8" t="str"/>
-      <x:c r="K9" s="8" t="str"/>
-      <x:c r="L9" s="8" t="str">
+        <x:v>Female/male TTS preference; actual availability depends on the installed Android voice engine.</x:v>
+      </x:c>
+      <x:c r="E9" s="8"/>
+      <x:c r="F9" s="8" t="str">
         <x:v>yes</x:v>
       </x:c>
-      <x:c r="M9" s="8" t="str"/>
+      <x:c r="G9" s="8"/>
+      <x:c r="H9" s="8"/>
+      <x:c r="I9" s="8"/>
+      <x:c r="J9" s="8"/>
+      <x:c r="K9" s="8" t="str">
+        <x:v>female</x:v>
+      </x:c>
+      <x:c r="L9" s="8"/>
+      <x:c r="M9" s="8"/>
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="8" t="str">
-        <x:v>text</x:v>
+        <x:v>select_one yes_no</x:v>
       </x:c>
       <x:c r="B10" s="8" t="str">
-        <x:v>conversation_transcript</x:v>
+        <x:v>spoken_output_input</x:v>
       </x:c>
       <x:c r="C10" s="8" t="str">
-        <x:v>Conversation transcript</x:v>
-      </x:c>
-      <x:c r="D10" s="8" t="str">
-        <x:v>Returned by MethodMesh.</x:v>
-      </x:c>
-      <x:c r="E10" s="8" t="str">
-        <x:v>hidden-answer</x:v>
-      </x:c>
-      <x:c r="F10" s="8" t="str"/>
-      <x:c r="G10" s="8" t="str"/>
-      <x:c r="H10" s="8" t="str"/>
-      <x:c r="I10" s="8" t="str"/>
-      <x:c r="J10" s="8" t="str"/>
-      <x:c r="K10" s="8" t="str"/>
+        <x:v>Speak translations aloud</x:v>
+      </x:c>
+      <x:c r="D10" s="8"/>
+      <x:c r="E10" s="8"/>
+      <x:c r="F10" s="8" t="str">
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="G10" s="8"/>
+      <x:c r="H10" s="8"/>
+      <x:c r="I10" s="8"/>
+      <x:c r="J10" s="8"/>
+      <x:c r="K10" s="8" t="str">
+        <x:v>true</x:v>
+      </x:c>
       <x:c r="L10" s="8" t="str">
         <x:v>yes</x:v>
       </x:c>
-      <x:c r="M10" s="8" t="str"/>
+      <x:c r="M10" s="8"/>
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="8" t="str">
-        <x:v>text</x:v>
+        <x:v>select_one yes_no</x:v>
       </x:c>
       <x:c r="B11" s="8" t="str">
-        <x:v>methodmesh_full_json</x:v>
+        <x:v>prefer_offline_input</x:v>
       </x:c>
       <x:c r="C11" s="8" t="str">
-        <x:v>MethodMesh metadata JSON</x:v>
-      </x:c>
-      <x:c r="D11" s="8" t="str">
-        <x:v>Shared MethodMesh FULL execution envelope. Retained for complete execution/audit capture; capability-specific return fields are projected separately.</x:v>
-      </x:c>
-      <x:c r="E11" s="8" t="str">
-        <x:v>hidden-answer</x:v>
-      </x:c>
-      <x:c r="F11" s="8" t="str"/>
-      <x:c r="G11" s="8" t="str"/>
-      <x:c r="H11" s="8" t="str"/>
-      <x:c r="I11" s="8" t="str"/>
-      <x:c r="J11" s="8" t="str"/>
-      <x:c r="K11" s="8" t="str"/>
+        <x:v>Prefer offline speech recognition</x:v>
+      </x:c>
+      <x:c r="D11" s="8"/>
+      <x:c r="E11" s="8"/>
+      <x:c r="F11" s="8" t="str">
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="G11" s="8"/>
+      <x:c r="H11" s="8"/>
+      <x:c r="I11" s="8"/>
+      <x:c r="J11" s="8"/>
+      <x:c r="K11" s="8" t="str">
+        <x:v>false</x:v>
+      </x:c>
       <x:c r="L11" s="8" t="str">
         <x:v>yes</x:v>
       </x:c>
-      <x:c r="M11" s="8" t="str"/>
+      <x:c r="M11" s="8"/>
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="8" t="str">
-        <x:v>end_group</x:v>
-      </x:c>
-      <x:c r="B12" s="8" t="str"/>
-      <x:c r="C12" s="8" t="str"/>
-      <x:c r="D12" s="8" t="str"/>
-      <x:c r="E12" s="8" t="str"/>
-      <x:c r="F12" s="8" t="str"/>
-      <x:c r="G12" s="8" t="str"/>
-      <x:c r="H12" s="8" t="str"/>
-      <x:c r="I12" s="8" t="str"/>
-      <x:c r="J12" s="8" t="str"/>
-      <x:c r="K12" s="8" t="str"/>
-      <x:c r="L12" s="8" t="str"/>
-      <x:c r="M12" s="8" t="str"/>
+        <x:v>select_one yes_no</x:v>
+      </x:c>
+      <x:c r="B12" s="8" t="str">
+        <x:v>transcript_on_start_input</x:v>
+      </x:c>
+      <x:c r="C12" s="8" t="str">
+        <x:v>Transcript on at start</x:v>
+      </x:c>
+      <x:c r="D12" s="8" t="str">
+        <x:v>Can be paused/resumed while translation continues.</x:v>
+      </x:c>
+      <x:c r="E12" s="8"/>
+      <x:c r="F12" s="8" t="str">
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="G12" s="8"/>
+      <x:c r="H12" s="8"/>
+      <x:c r="I12" s="8"/>
+      <x:c r="J12" s="8"/>
+      <x:c r="K12" s="8" t="str">
+        <x:v>true</x:v>
+      </x:c>
+      <x:c r="L12" s="8" t="str">
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="M12" s="8"/>
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="8" t="str">
+        <x:v>text</x:v>
+      </x:c>
+      <x:c r="B13" s="8" t="str">
+        <x:v>methodmesh_execution_id</x:v>
+      </x:c>
+      <x:c r="C13" s="8" t="str">
+        <x:v>MethodMesh execution ID</x:v>
+      </x:c>
+      <x:c r="D13" s="8" t="str">
+        <x:v>Returned by MethodMesh.</x:v>
+      </x:c>
+      <x:c r="E13" s="8" t="str">
+        <x:v>hidden-answer</x:v>
+      </x:c>
+      <x:c r="F13" s="8"/>
+      <x:c r="G13" s="8"/>
+      <x:c r="H13" s="8"/>
+      <x:c r="I13" s="8"/>
+      <x:c r="J13" s="8"/>
+      <x:c r="K13" s="8"/>
+      <x:c r="L13" s="8" t="str">
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="M13" s="8"/>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" t="str">
+        <x:v>text</x:v>
+      </x:c>
+      <x:c r="B14" t="str">
+        <x:v>methodmesh_status</x:v>
+      </x:c>
+      <x:c r="C14" t="str">
+        <x:v>MethodMesh status</x:v>
+      </x:c>
+      <x:c r="D14" t="str">
+        <x:v>Shared transport status.</x:v>
+      </x:c>
+      <x:c r="E14" t="str">
+        <x:v>hidden-answer</x:v>
+      </x:c>
+      <x:c r="F14"/>
+      <x:c r="G14"/>
+      <x:c r="H14"/>
+      <x:c r="I14"/>
+      <x:c r="J14"/>
+      <x:c r="K14"/>
+      <x:c r="L14"/>
+      <x:c r="M14"/>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" t="str">
+        <x:v>text</x:v>
+      </x:c>
+      <x:c r="B15" t="str">
+        <x:v>conversation_transcript</x:v>
+      </x:c>
+      <x:c r="C15" t="str">
+        <x:v>Conversation transcript</x:v>
+      </x:c>
+      <x:c r="D15" t="str">
+        <x:v>Includes pause/resume break markers.</x:v>
+      </x:c>
+      <x:c r="E15" t="str">
+        <x:v>hidden-answer</x:v>
+      </x:c>
+      <x:c r="F15"/>
+      <x:c r="G15"/>
+      <x:c r="H15"/>
+      <x:c r="I15"/>
+      <x:c r="J15"/>
+      <x:c r="K15"/>
+      <x:c r="L15"/>
+      <x:c r="M15"/>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" t="str">
+        <x:v>text</x:v>
+      </x:c>
+      <x:c r="B16" t="str">
+        <x:v>methodmesh_full_json</x:v>
+      </x:c>
+      <x:c r="C16" t="str">
+        <x:v>MethodMesh metadata JSON</x:v>
+      </x:c>
+      <x:c r="D16" t="str">
+        <x:v>FULL envelope including turn/event data.</x:v>
+      </x:c>
+      <x:c r="E16" t="str">
+        <x:v>hidden-answer</x:v>
+      </x:c>
+      <x:c r="F16"/>
+      <x:c r="G16"/>
+      <x:c r="H16"/>
+      <x:c r="I16"/>
+      <x:c r="J16"/>
+      <x:c r="K16"/>
+      <x:c r="L16"/>
+      <x:c r="M16"/>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" t="str">
+        <x:v>end_group</x:v>
+      </x:c>
+      <x:c r="B17"/>
+      <x:c r="C17"/>
+      <x:c r="D17"/>
+      <x:c r="E17"/>
+      <x:c r="F17"/>
+      <x:c r="G17"/>
+      <x:c r="H17"/>
+      <x:c r="I17"/>
+      <x:c r="J17"/>
+      <x:c r="K17"/>
+      <x:c r="L17"/>
+      <x:c r="M17"/>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" t="str">
         <x:v>note</x:v>
       </x:c>
-      <x:c r="B13" s="8" t="str">
+      <x:c r="B18" t="str">
         <x:v>return_summary</x:v>
       </x:c>
-      <x:c r="C13" s="8" t="str">
+      <x:c r="C18" t="str">
         <x:v>MethodMesh return captured. Status: ${methodmesh_status}</x:v>
       </x:c>
-      <x:c r="D13" s="8" t="str">
-        <x:v>Only fields relevant to this capability are stored, plus the shared FULL envelope.</x:v>
-      </x:c>
-      <x:c r="E13" s="8" t="str"/>
-      <x:c r="F13" s="8" t="str"/>
-      <x:c r="G13" s="8" t="str"/>
-      <x:c r="H13" s="8" t="str"/>
-      <x:c r="I13" s="8" t="str"/>
-      <x:c r="J13" s="8" t="str"/>
-      <x:c r="K13" s="8" t="str"/>
-      <x:c r="L13" s="8" t="str"/>
-      <x:c r="M13" s="8" t="str"/>
+      <x:c r="D18"/>
+      <x:c r="E18"/>
+      <x:c r="F18"/>
+      <x:c r="G18"/>
+      <x:c r="H18"/>
+      <x:c r="I18"/>
+      <x:c r="J18"/>
+      <x:c r="K18"/>
+      <x:c r="L18"/>
+      <x:c r="M18"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -634,9 +772,9 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="24" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="24" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="40" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="14" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="10" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="28" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">
@@ -655,10 +793,10 @@
         <x:v>language</x:v>
       </x:c>
       <x:c r="B2" s="8" t="str">
-        <x:v>en</x:v>
+        <x:v>af</x:v>
       </x:c>
       <x:c r="C2" s="8" t="str">
-        <x:v>English (En)</x:v>
+        <x:v>Afrikaans (Af)</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -666,10 +804,10 @@
         <x:v>language</x:v>
       </x:c>
       <x:c r="B3" s="8" t="str">
-        <x:v>es</x:v>
+        <x:v>sq</x:v>
       </x:c>
       <x:c r="C3" s="8" t="str">
-        <x:v>Spanish (Es)</x:v>
+        <x:v>Albanian (Sq)</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
@@ -677,10 +815,10 @@
         <x:v>language</x:v>
       </x:c>
       <x:c r="B4" s="8" t="str">
-        <x:v>fr</x:v>
+        <x:v>ar</x:v>
       </x:c>
       <x:c r="C4" s="8" t="str">
-        <x:v>French (Fr)</x:v>
+        <x:v>Arabic (Ar)</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
@@ -688,10 +826,10 @@
         <x:v>language</x:v>
       </x:c>
       <x:c r="B5" s="8" t="str">
-        <x:v>pt</x:v>
+        <x:v>be</x:v>
       </x:c>
       <x:c r="C5" s="8" t="str">
-        <x:v>Portuguese (Pt)</x:v>
+        <x:v>Belarusian (Be)</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -699,10 +837,10 @@
         <x:v>language</x:v>
       </x:c>
       <x:c r="B6" s="8" t="str">
-        <x:v>de</x:v>
+        <x:v>bn</x:v>
       </x:c>
       <x:c r="C6" s="8" t="str">
-        <x:v>German (De)</x:v>
+        <x:v>Bengali (Bn)</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -710,10 +848,10 @@
         <x:v>language</x:v>
       </x:c>
       <x:c r="B7" s="8" t="str">
-        <x:v>it</x:v>
+        <x:v>bg</x:v>
       </x:c>
       <x:c r="C7" s="8" t="str">
-        <x:v>Italian (It)</x:v>
+        <x:v>Bulgarian (Bg)</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -721,10 +859,10 @@
         <x:v>language</x:v>
       </x:c>
       <x:c r="B8" s="8" t="str">
-        <x:v>ar</x:v>
+        <x:v>ca</x:v>
       </x:c>
       <x:c r="C8" s="8" t="str">
-        <x:v>Arabic (Ar)</x:v>
+        <x:v>Catalan (Ca)</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -732,10 +870,10 @@
         <x:v>language</x:v>
       </x:c>
       <x:c r="B9" s="8" t="str">
-        <x:v>hi</x:v>
+        <x:v>zh</x:v>
       </x:c>
       <x:c r="C9" s="8" t="str">
-        <x:v>Hindi (Hi)</x:v>
+        <x:v>Chinese (Zh)</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -743,10 +881,10 @@
         <x:v>language</x:v>
       </x:c>
       <x:c r="B10" s="8" t="str">
-        <x:v>sw</x:v>
+        <x:v>hr</x:v>
       </x:c>
       <x:c r="C10" s="8" t="str">
-        <x:v>Swahili (Sw)</x:v>
+        <x:v>Croatian (Hr)</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
@@ -754,10 +892,10 @@
         <x:v>language</x:v>
       </x:c>
       <x:c r="B11" s="8" t="str">
-        <x:v>zh</x:v>
+        <x:v>cs</x:v>
       </x:c>
       <x:c r="C11" s="8" t="str">
-        <x:v>Chinese (Zh)</x:v>
+        <x:v>Czech (Cs)</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
@@ -765,32 +903,615 @@
         <x:v>language</x:v>
       </x:c>
       <x:c r="B12" s="8" t="str">
-        <x:v>kri</x:v>
+        <x:v>da</x:v>
       </x:c>
       <x:c r="C12" s="8" t="str">
-        <x:v>Krio (Kri) — if supported by installed translation engine</x:v>
+        <x:v>Danish (Da)</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="8" t="str">
-        <x:v>yes_no</x:v>
+        <x:v>language</x:v>
       </x:c>
       <x:c r="B13" s="8" t="str">
-        <x:v>true</x:v>
+        <x:v>nl</x:v>
       </x:c>
       <x:c r="C13" s="8" t="str">
-        <x:v>Yes</x:v>
+        <x:v>Dutch (Nl)</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="8" t="str">
+        <x:v>language</x:v>
+      </x:c>
+      <x:c r="B14" s="8" t="str">
+        <x:v>en</x:v>
+      </x:c>
+      <x:c r="C14" s="8" t="str">
+        <x:v>English (En)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" s="8" t="str">
+        <x:v>language</x:v>
+      </x:c>
+      <x:c r="B15" s="8" t="str">
+        <x:v>eo</x:v>
+      </x:c>
+      <x:c r="C15" s="8" t="str">
+        <x:v>Esperanto (Eo)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" s="8" t="str">
+        <x:v>language</x:v>
+      </x:c>
+      <x:c r="B16" s="8" t="str">
+        <x:v>et</x:v>
+      </x:c>
+      <x:c r="C16" s="8" t="str">
+        <x:v>Estonian (Et)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" s="8" t="str">
+        <x:v>language</x:v>
+      </x:c>
+      <x:c r="B17" s="8" t="str">
+        <x:v>fi</x:v>
+      </x:c>
+      <x:c r="C17" s="8" t="str">
+        <x:v>Finnish (Fi)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" s="8" t="str">
+        <x:v>language</x:v>
+      </x:c>
+      <x:c r="B18" s="8" t="str">
+        <x:v>fr</x:v>
+      </x:c>
+      <x:c r="C18" s="8" t="str">
+        <x:v>French (Fr)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" s="8" t="str">
+        <x:v>language</x:v>
+      </x:c>
+      <x:c r="B19" s="8" t="str">
+        <x:v>gl</x:v>
+      </x:c>
+      <x:c r="C19" s="8" t="str">
+        <x:v>Galician (Gl)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" s="8" t="str">
+        <x:v>language</x:v>
+      </x:c>
+      <x:c r="B20" s="8" t="str">
+        <x:v>ka</x:v>
+      </x:c>
+      <x:c r="C20" s="8" t="str">
+        <x:v>Georgian (Ka)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" s="8" t="str">
+        <x:v>language</x:v>
+      </x:c>
+      <x:c r="B21" s="8" t="str">
+        <x:v>de</x:v>
+      </x:c>
+      <x:c r="C21" s="8" t="str">
+        <x:v>German (De)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" s="8" t="str">
+        <x:v>language</x:v>
+      </x:c>
+      <x:c r="B22" s="8" t="str">
+        <x:v>el</x:v>
+      </x:c>
+      <x:c r="C22" s="8" t="str">
+        <x:v>Greek (El)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23">
+      <x:c r="A23" s="8" t="str">
+        <x:v>language</x:v>
+      </x:c>
+      <x:c r="B23" s="8" t="str">
+        <x:v>gu</x:v>
+      </x:c>
+      <x:c r="C23" s="8" t="str">
+        <x:v>Gujarati (Gu)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24">
+      <x:c r="A24" s="8" t="str">
+        <x:v>language</x:v>
+      </x:c>
+      <x:c r="B24" s="8" t="str">
+        <x:v>ht</x:v>
+      </x:c>
+      <x:c r="C24" s="8" t="str">
+        <x:v>Haitian Creole (Ht)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25">
+      <x:c r="A25" s="8" t="str">
+        <x:v>language</x:v>
+      </x:c>
+      <x:c r="B25" s="8" t="str">
+        <x:v>he</x:v>
+      </x:c>
+      <x:c r="C25" s="8" t="str">
+        <x:v>Hebrew (He)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26">
+      <x:c r="A26" s="8" t="str">
+        <x:v>language</x:v>
+      </x:c>
+      <x:c r="B26" s="8" t="str">
+        <x:v>hi</x:v>
+      </x:c>
+      <x:c r="C26" s="8" t="str">
+        <x:v>Hindi (Hi)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27">
+      <x:c r="A27" s="8" t="str">
+        <x:v>language</x:v>
+      </x:c>
+      <x:c r="B27" s="8" t="str">
+        <x:v>hu</x:v>
+      </x:c>
+      <x:c r="C27" s="8" t="str">
+        <x:v>Hungarian (Hu)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28">
+      <x:c r="A28" s="8" t="str">
+        <x:v>language</x:v>
+      </x:c>
+      <x:c r="B28" s="8" t="str">
+        <x:v>is</x:v>
+      </x:c>
+      <x:c r="C28" s="8" t="str">
+        <x:v>Icelandic (Is)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29">
+      <x:c r="A29" s="8" t="str">
+        <x:v>language</x:v>
+      </x:c>
+      <x:c r="B29" s="8" t="str">
+        <x:v>id</x:v>
+      </x:c>
+      <x:c r="C29" s="8" t="str">
+        <x:v>Indonesian (Id)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30">
+      <x:c r="A30" s="8" t="str">
+        <x:v>language</x:v>
+      </x:c>
+      <x:c r="B30" s="8" t="str">
+        <x:v>ga</x:v>
+      </x:c>
+      <x:c r="C30" s="8" t="str">
+        <x:v>Irish (Ga)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="31">
+      <x:c r="A31" s="8" t="str">
+        <x:v>language</x:v>
+      </x:c>
+      <x:c r="B31" s="8" t="str">
+        <x:v>it</x:v>
+      </x:c>
+      <x:c r="C31" s="8" t="str">
+        <x:v>Italian (It)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="32">
+      <x:c r="A32" s="8" t="str">
+        <x:v>language</x:v>
+      </x:c>
+      <x:c r="B32" s="8" t="str">
+        <x:v>ja</x:v>
+      </x:c>
+      <x:c r="C32" s="8" t="str">
+        <x:v>Japanese (Ja)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="33">
+      <x:c r="A33" s="8" t="str">
+        <x:v>language</x:v>
+      </x:c>
+      <x:c r="B33" s="8" t="str">
+        <x:v>kn</x:v>
+      </x:c>
+      <x:c r="C33" s="8" t="str">
+        <x:v>Kannada (Kn)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="34">
+      <x:c r="A34" s="8" t="str">
+        <x:v>language</x:v>
+      </x:c>
+      <x:c r="B34" s="8" t="str">
+        <x:v>ko</x:v>
+      </x:c>
+      <x:c r="C34" s="8" t="str">
+        <x:v>Korean (Ko)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="35">
+      <x:c r="A35" s="8" t="str">
+        <x:v>language</x:v>
+      </x:c>
+      <x:c r="B35" s="8" t="str">
+        <x:v>lv</x:v>
+      </x:c>
+      <x:c r="C35" s="8" t="str">
+        <x:v>Latvian (Lv)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="36">
+      <x:c r="A36" s="8" t="str">
+        <x:v>language</x:v>
+      </x:c>
+      <x:c r="B36" s="8" t="str">
+        <x:v>lt</x:v>
+      </x:c>
+      <x:c r="C36" s="8" t="str">
+        <x:v>Lithuanian (Lt)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="37">
+      <x:c r="A37" s="8" t="str">
+        <x:v>language</x:v>
+      </x:c>
+      <x:c r="B37" s="8" t="str">
+        <x:v>mk</x:v>
+      </x:c>
+      <x:c r="C37" s="8" t="str">
+        <x:v>Macedonian (Mk)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="38">
+      <x:c r="A38" s="8" t="str">
+        <x:v>language</x:v>
+      </x:c>
+      <x:c r="B38" s="8" t="str">
+        <x:v>ms</x:v>
+      </x:c>
+      <x:c r="C38" s="8" t="str">
+        <x:v>Malay (Ms)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="39">
+      <x:c r="A39" s="8" t="str">
+        <x:v>language</x:v>
+      </x:c>
+      <x:c r="B39" s="8" t="str">
+        <x:v>mt</x:v>
+      </x:c>
+      <x:c r="C39" s="8" t="str">
+        <x:v>Maltese (Mt)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="40">
+      <x:c r="A40" s="8" t="str">
+        <x:v>language</x:v>
+      </x:c>
+      <x:c r="B40" s="8" t="str">
+        <x:v>mr</x:v>
+      </x:c>
+      <x:c r="C40" s="8" t="str">
+        <x:v>Marathi (Mr)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="41">
+      <x:c r="A41" s="8" t="str">
+        <x:v>language</x:v>
+      </x:c>
+      <x:c r="B41" s="8" t="str">
+        <x:v>no</x:v>
+      </x:c>
+      <x:c r="C41" s="8" t="str">
+        <x:v>Norwegian (No)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="42">
+      <x:c r="A42" s="8" t="str">
+        <x:v>language</x:v>
+      </x:c>
+      <x:c r="B42" s="8" t="str">
+        <x:v>fa</x:v>
+      </x:c>
+      <x:c r="C42" s="8" t="str">
+        <x:v>Persian (Fa)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="43">
+      <x:c r="A43" s="8" t="str">
+        <x:v>language</x:v>
+      </x:c>
+      <x:c r="B43" s="8" t="str">
+        <x:v>pl</x:v>
+      </x:c>
+      <x:c r="C43" s="8" t="str">
+        <x:v>Polish (Pl)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="44">
+      <x:c r="A44" s="8" t="str">
+        <x:v>language</x:v>
+      </x:c>
+      <x:c r="B44" s="8" t="str">
+        <x:v>pt</x:v>
+      </x:c>
+      <x:c r="C44" s="8" t="str">
+        <x:v>Portuguese (Pt)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="45">
+      <x:c r="A45" s="8" t="str">
+        <x:v>language</x:v>
+      </x:c>
+      <x:c r="B45" s="8" t="str">
+        <x:v>ro</x:v>
+      </x:c>
+      <x:c r="C45" s="8" t="str">
+        <x:v>Romanian (Ro)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="46">
+      <x:c r="A46" s="8" t="str">
+        <x:v>language</x:v>
+      </x:c>
+      <x:c r="B46" s="8" t="str">
+        <x:v>ru</x:v>
+      </x:c>
+      <x:c r="C46" s="8" t="str">
+        <x:v>Russian (Ru)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="47">
+      <x:c r="A47" s="8" t="str">
+        <x:v>language</x:v>
+      </x:c>
+      <x:c r="B47" s="8" t="str">
+        <x:v>sk</x:v>
+      </x:c>
+      <x:c r="C47" s="8" t="str">
+        <x:v>Slovak (Sk)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="48">
+      <x:c r="A48" s="8" t="str">
+        <x:v>language</x:v>
+      </x:c>
+      <x:c r="B48" s="8" t="str">
+        <x:v>sl</x:v>
+      </x:c>
+      <x:c r="C48" s="8" t="str">
+        <x:v>Slovenian (Sl)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="49">
+      <x:c r="A49" s="8" t="str">
+        <x:v>language</x:v>
+      </x:c>
+      <x:c r="B49" s="8" t="str">
+        <x:v>es</x:v>
+      </x:c>
+      <x:c r="C49" s="8" t="str">
+        <x:v>Spanish (Es)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="50">
+      <x:c r="A50" s="8" t="str">
+        <x:v>language</x:v>
+      </x:c>
+      <x:c r="B50" s="8" t="str">
+        <x:v>sw</x:v>
+      </x:c>
+      <x:c r="C50" s="8" t="str">
+        <x:v>Swahili (Sw)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="51">
+      <x:c r="A51" s="8" t="str">
+        <x:v>language</x:v>
+      </x:c>
+      <x:c r="B51" s="8" t="str">
+        <x:v>sv</x:v>
+      </x:c>
+      <x:c r="C51" s="8" t="str">
+        <x:v>Swedish (Sv)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="52">
+      <x:c r="A52" s="8" t="str">
+        <x:v>language</x:v>
+      </x:c>
+      <x:c r="B52" s="8" t="str">
+        <x:v>tl</x:v>
+      </x:c>
+      <x:c r="C52" s="8" t="str">
+        <x:v>Tagalog (Tl)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="53">
+      <x:c r="A53" s="8" t="str">
+        <x:v>language</x:v>
+      </x:c>
+      <x:c r="B53" s="8" t="str">
+        <x:v>ta</x:v>
+      </x:c>
+      <x:c r="C53" s="8" t="str">
+        <x:v>Tamil (Ta)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="54">
+      <x:c r="A54" s="8" t="str">
+        <x:v>language</x:v>
+      </x:c>
+      <x:c r="B54" s="8" t="str">
+        <x:v>te</x:v>
+      </x:c>
+      <x:c r="C54" s="8" t="str">
+        <x:v>Telugu (Te)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="55">
+      <x:c r="A55" s="8" t="str">
+        <x:v>language</x:v>
+      </x:c>
+      <x:c r="B55" s="8" t="str">
+        <x:v>th</x:v>
+      </x:c>
+      <x:c r="C55" s="8" t="str">
+        <x:v>Thai (Th)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="56">
+      <x:c r="A56" s="8" t="str">
+        <x:v>language</x:v>
+      </x:c>
+      <x:c r="B56" s="8" t="str">
+        <x:v>tr</x:v>
+      </x:c>
+      <x:c r="C56" s="8" t="str">
+        <x:v>Turkish (Tr)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="57">
+      <x:c r="A57" s="8" t="str">
+        <x:v>language</x:v>
+      </x:c>
+      <x:c r="B57" s="8" t="str">
+        <x:v>uk</x:v>
+      </x:c>
+      <x:c r="C57" s="8" t="str">
+        <x:v>Ukrainian (Uk)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="58">
+      <x:c r="A58" s="8" t="str">
+        <x:v>language</x:v>
+      </x:c>
+      <x:c r="B58" s="8" t="str">
+        <x:v>ur</x:v>
+      </x:c>
+      <x:c r="C58" s="8" t="str">
+        <x:v>Urdu (Ur)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="59">
+      <x:c r="A59" s="8" t="str">
+        <x:v>language</x:v>
+      </x:c>
+      <x:c r="B59" s="8" t="str">
+        <x:v>vi</x:v>
+      </x:c>
+      <x:c r="C59" s="8" t="str">
+        <x:v>Vietnamese (Vi)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="60">
+      <x:c r="A60" s="8" t="str">
+        <x:v>language</x:v>
+      </x:c>
+      <x:c r="B60" s="8" t="str">
+        <x:v>cy</x:v>
+      </x:c>
+      <x:c r="C60" s="8" t="str">
+        <x:v>Welsh (Cy)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="61">
+      <x:c r="A61" s="8" t="str">
         <x:v>yes_no</x:v>
       </x:c>
-      <x:c r="B14" s="8" t="str">
+      <x:c r="B61" s="8" t="str">
+        <x:v>true</x:v>
+      </x:c>
+      <x:c r="C61" s="8" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="62">
+      <x:c r="A62" s="8" t="str">
+        <x:v>yes_no</x:v>
+      </x:c>
+      <x:c r="B62" s="8" t="str">
         <x:v>false</x:v>
       </x:c>
-      <x:c r="C14" s="8" t="str">
+      <x:c r="C62" s="8" t="str">
         <x:v>No</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="63">
+      <x:c r="A63" t="str">
+        <x:v>arabic_variant</x:v>
+      </x:c>
+      <x:c r="B63" t="str">
+        <x:v>levantine</x:v>
+      </x:c>
+      <x:c r="C63" t="str">
+        <x:v>Levantine · الشامية</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="64">
+      <x:c r="A64" t="str">
+        <x:v>arabic_variant</x:v>
+      </x:c>
+      <x:c r="B64" t="str">
+        <x:v>gulf</x:v>
+      </x:c>
+      <x:c r="C64" t="str">
+        <x:v>Gulf · الخليجية</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="65">
+      <x:c r="A65" t="str">
+        <x:v>arabic_variant</x:v>
+      </x:c>
+      <x:c r="B65" t="str">
+        <x:v>north_african</x:v>
+      </x:c>
+      <x:c r="C65" t="str">
+        <x:v>North African · شمال أفريقيا</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="66">
+      <x:c r="A66" t="str">
+        <x:v>voice_preference</x:v>
+      </x:c>
+      <x:c r="B66" t="str">
+        <x:v>female</x:v>
+      </x:c>
+      <x:c r="C66" t="str">
+        <x:v>Female ♀</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="67">
+      <x:c r="A67" t="str">
+        <x:v>voice_preference</x:v>
+      </x:c>
+      <x:c r="B67" t="str">
+        <x:v>male</x:v>
+      </x:c>
+      <x:c r="C67" t="str">
+        <x:v>Male ♂</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -826,8 +1547,13 @@
         <x:v>conversationtranslate_conversation_translate</x:v>
       </x:c>
       <x:c r="C2" t="str">
-        <x:v>2026090701</x:v>
-      </x:c>
+        <x:v>2026091102</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3"/>
+      <x:c r="B3"/>
+      <x:c r="C3"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>